<commit_message>
Expand ETL package with dimension loads
Adds SQL-to-Excel data flows for additional airline dimensions, updates package metadata and project version, and refreshes the Excel output workbook.
</commit_message>
<xml_diff>
--- a/HC/BDAeroLineas.xlsx
+++ b/HC/BDAeroLineas.xlsx
@@ -9,11 +9,17 @@
   <sheets>
     <sheet sheetId="1" r:id="rId1" name="Hoja1"/>
     <sheet r:id="rId4" sheetId="2" name="DimAeronave"/>
-    <sheet r:id="rId5" name="DimAeropuerto" sheetId="3"/>
+    <sheet r:id="rId5" sheetId="3" name="DimAeropuerto"/>
+    <sheet r:id="rId6" sheetId="4" name="DimCausaDemora"/>
+    <sheet r:id="rId7" sheetId="5" name="DimClima"/>
+    <sheet r:id="rId8" name="DimEstadoVuelo" sheetId="6"/>
   </sheets>
   <definedNames>
     <definedName name="DimAeronave">'DimAeronave'!$A$1:$E$1</definedName>
     <definedName name="DimAeropuerto">'DimAeropuerto'!$A$1:$F$1</definedName>
+    <definedName name="DimCausaDemora">'DimCausaDemora'!$A$1:$D$1</definedName>
+    <definedName name="DimClima">'DimClima'!$A$1:$F$1</definedName>
+    <definedName name="DimEstadoVuelo">'DimEstadoVuelo'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="true"/>
   <extLst>
@@ -421,4 +427,110 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdCausaPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>DescripcionCausa</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>CategoriaCausa</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>AplicaIndemnizacion</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdClimaPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>VelocidadVientoKmh</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>VisibilidadMetros</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>PrecipitacionMm</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>TemperaturaGradosC</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>PresionAtmosfericaHpa</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdEstadoPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>NumeroVuelo</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>EstadoOperacion</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>NivelImpactoItinerario</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand SSIS dimension exports
Adds ETL sources and Excel destinations for additional dimensions, updates the Excel connection settings and workbook, and disables sensitive-value persistence in the SSIS project.
</commit_message>
<xml_diff>
--- a/HC/BDAeroLineas.xlsx
+++ b/HC/BDAeroLineas.xlsx
@@ -12,7 +12,9 @@
     <sheet r:id="rId5" sheetId="3" name="DimAeropuerto"/>
     <sheet r:id="rId6" sheetId="4" name="DimCausaDemora"/>
     <sheet r:id="rId7" sheetId="5" name="DimClima"/>
-    <sheet r:id="rId8" name="DimEstadoVuelo" sheetId="6"/>
+    <sheet r:id="rId8" sheetId="6" name="DimEstadoVuelo"/>
+    <sheet r:id="rId9" sheetId="7" name="DimFenomenoClimatico"/>
+    <sheet r:id="rId10" name="DimRuta" sheetId="8"/>
   </sheets>
   <definedNames>
     <definedName name="DimAeronave">'DimAeronave'!$A$1:$E$1</definedName>
@@ -20,6 +22,8 @@
     <definedName name="DimCausaDemora">'DimCausaDemora'!$A$1:$D$1</definedName>
     <definedName name="DimClima">'DimClima'!$A$1:$F$1</definedName>
     <definedName name="DimEstadoVuelo">'DimEstadoVuelo'!$A$1:$D$1</definedName>
+    <definedName name="DimFenomenoClimatico">'DimFenomenoClimatico'!$A$1:$D$1</definedName>
+    <definedName name="DimRuta">'DimRuta'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="true"/>
   <extLst>
@@ -533,4 +537,78 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdFenomenoPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>NombreFenomeno</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>TipoAnomalia</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>NivelSeveridad</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdRutaPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>CodigoRuta</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>CiudadOrigen</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>CiudadDestino</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>DistanciaKm</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>DuracionMin</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Completito para el MR HuATAY
</commit_message>
<xml_diff>
--- a/HC/BDAeroLineas.xlsx
+++ b/HC/BDAeroLineas.xlsx
@@ -14,7 +14,10 @@
     <sheet r:id="rId7" sheetId="5" name="DimClima"/>
     <sheet r:id="rId8" sheetId="6" name="DimEstadoVuelo"/>
     <sheet r:id="rId9" sheetId="7" name="DimFenomenoClimatico"/>
-    <sheet r:id="rId10" name="DimRuta" sheetId="8"/>
+    <sheet r:id="rId10" sheetId="8" name="DimRuta"/>
+    <sheet r:id="rId11" sheetId="9" name="DimTiempo"/>
+    <sheet r:id="rId12" sheetId="10" name="DimTripulacion"/>
+    <sheet r:id="rId13" name="FactDemoraVuelo" sheetId="11"/>
   </sheets>
   <definedNames>
     <definedName name="DimAeronave">'DimAeronave'!$A$1:$E$1</definedName>
@@ -24,6 +27,9 @@
     <definedName name="DimEstadoVuelo">'DimEstadoVuelo'!$A$1:$D$1</definedName>
     <definedName name="DimFenomenoClimatico">'DimFenomenoClimatico'!$A$1:$D$1</definedName>
     <definedName name="DimRuta">'DimRuta'!$A$1:$F$1</definedName>
+    <definedName name="DimTiempo">'DimTiempo'!$A$1:$H$1</definedName>
+    <definedName name="DimTripulacion">'DimTripulacion'!$A$1:$F$1</definedName>
+    <definedName name="FactDemoraVuelo">'FactDemoraVuelo'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="true"/>
   <extLst>
@@ -354,6 +360,145 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdTripulacionPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>CodigoEquipo</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>CapitanCargo</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>HorasVueloAcumuladas</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>NivelFatiga</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>TurnoOperativo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdHechoDemoraPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>IdTiempoFK</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>IdAeropuertoFK</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>IdRutaFK</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>IdAeronaveFK</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>IdTripulacionFK</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>IdClimaFK</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>IdFenomenoFK</t>
+        </is>
+      </c>
+      <c r="I1" s="0" t="inlineStr">
+        <is>
+          <t>IdCausaFK</t>
+        </is>
+      </c>
+      <c r="J1" s="0" t="inlineStr">
+        <is>
+          <t>IdEstadoFK</t>
+        </is>
+      </c>
+      <c r="K1" s="0" t="inlineStr">
+        <is>
+          <t>MinutosRetrasoSalida</t>
+        </is>
+      </c>
+      <c r="L1" s="0" t="inlineStr">
+        <is>
+          <t>MinutosRetrasoLlegada</t>
+        </is>
+      </c>
+      <c r="M1" s="0" t="inlineStr">
+        <is>
+          <t>MinutosRetrasoAcumulados</t>
+        </is>
+      </c>
+      <c r="N1" s="0" t="inlineStr">
+        <is>
+          <t>CombustibleConsumidoGal</t>
+        </is>
+      </c>
+      <c r="O1" s="0" t="inlineStr">
+        <is>
+          <t>CostoOperativoAdicionalUSD</t>
+        </is>
+      </c>
+      <c r="P1" s="0" t="inlineStr">
+        <is>
+          <t>MontoIndemnizacionUSD</t>
+        </is>
+      </c>
+      <c r="Q1" s="0" t="inlineStr">
+        <is>
+          <t>PasajerosAfectados</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
@@ -611,4 +756,56 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row outlineLevel="0" r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>IdTiempoPK</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>Anio</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>Trimestre</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>DiaSemana</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>EstacionAnio</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>FranjaHoraria</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>